<commit_message>
test: 부하 테스트 (Locust) — REQ 평가 5-1 통과
설정:
- locust dev 의존성 추가
- seed_load_test_users.py: 50명 부하용 사용자 + 검진 + 챌린지 2건 + 체크인 10회
- tests/load/locustfile.py: 로그인 후 대시보드·챌린지·게이미피케이션 GET 12종 가중치 호출

결과 (동시 50명, 3분, 4,293 요청):
- ✅ API P95 = 18 ms (목표 3,000 ms, 0.6% 수준)
- P50 = 9 ms, P99 = 9,000 ms (POST /auth/login만 해당, bcrypt 비용)
- 실패율 0.00%
- GET API 12종 모두 P95 < 21 ms

산출물:
- docs/load-test/README.md — 평가용 보고서
- report.html / result_*.csv는 .gitignore 처리 (재생성 가능)

xlsx 갱신:
- REQ-NF-002 페이지 로딩 시간 → 완료 (실측 P95 18ms 부기)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/요구사항_정의서_v1.0_CKD.xlsx
+++ b/docs/요구사항_정의서_v1.0_CKD.xlsx
@@ -2083,8 +2083,8 @@
   <mergeCells count="4">
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>3초 이내</t>
+          <t>3초 이내 (실측 P95 18ms, 2026-06-01 부하 테스트)</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>대기중</t>
+          <t>완료</t>
         </is>
       </c>
     </row>

</xml_diff>